<commit_message>
13.09.2026 - PCB Mechanical Checks & 3D Validation
Continued working on the physical PCB layout and checking whether the component arrangement would actually work mechanically.
</commit_message>
<xml_diff>
--- a/Keyboard BOM.xlsx
+++ b/Keyboard BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ac8f2ab3c324b6b/Documents/GitHub/Crazy-75/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57AED7F5-C1AE-439E-BAFC-F0568EF62BD8}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46B8528B-391A-47F4-9DBB-EC9F55D9AE74}"/>
   <bookViews>
     <workbookView xWindow="24045" yWindow="4665" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t>Part No.</t>
   </si>
@@ -141,6 +141,21 @@
   </si>
   <si>
     <t>Screw-in scabilizers</t>
+  </si>
+  <si>
+    <t>USB cable</t>
+  </si>
+  <si>
+    <t>https://fr.aliexpress.com/item/1005005488898046.html?spm=a2g0o.productlist.main.4.748bKRxGKRxGnD&amp;aem_p4p_detail=20260912085948577072255597880000865035&amp;algo_pvid=6b40d4d7-b2a8-4461-84d5-216aaf7d8a13&amp;algo_exp_id=6b40d4d7-b2a8-4461-84d5-216aaf7d8a13-3&amp;pdp_ext_f=%7B%22order%22%3A%22896%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%211.26%211.26%21%21%211.43%211.43%21%400bafc98f17892287878784776e0d44%2112000033281493430%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3Ae8fc6401%3Bm03_new_user%3A-29895&amp;curPageLogUid=YTv5du2zwR8B&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005005488898046%7C_p_origin_prod%3A&amp;search_p4p_id=20260912085948577072255597880000865035_1</t>
+  </si>
+  <si>
+    <t>2.54mm PCB Pin headers</t>
+  </si>
+  <si>
+    <t>20x2p</t>
+  </si>
+  <si>
+    <t>25x2p</t>
   </si>
 </sst>
 </file>
@@ -523,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5F0154-0866-430C-ACD5-87E79D9222E2}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -787,6 +802,40 @@
         <v>6</v>
       </c>
     </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13">
+        <v>1.04</v>
+      </c>
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
24+26.09.2026 - Plate design
</commit_message>
<xml_diff>
--- a/Keyboard BOM.xlsx
+++ b/Keyboard BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ac8f2ab3c324b6b/Documents/GitHub/Crazy-75/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46B8528B-391A-47F4-9DBB-EC9F55D9AE74}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CBF6BE5-0C6D-49F8-BE6B-15503DDA57F8}"/>
   <bookViews>
-    <workbookView xWindow="24045" yWindow="4665" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
+    <workbookView xWindow="20775" yWindow="4425" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
   <si>
     <t>Part No.</t>
   </si>
@@ -144,18 +144,6 @@
   </si>
   <si>
     <t>USB cable</t>
-  </si>
-  <si>
-    <t>https://fr.aliexpress.com/item/1005005488898046.html?spm=a2g0o.productlist.main.4.748bKRxGKRxGnD&amp;aem_p4p_detail=20260912085948577072255597880000865035&amp;algo_pvid=6b40d4d7-b2a8-4461-84d5-216aaf7d8a13&amp;algo_exp_id=6b40d4d7-b2a8-4461-84d5-216aaf7d8a13-3&amp;pdp_ext_f=%7B%22order%22%3A%22896%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%211.26%211.26%21%21%211.43%211.43%21%400bafc98f17892287878784776e0d44%2112000033281493430%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3Ae8fc6401%3Bm03_new_user%3A-29895&amp;curPageLogUid=YTv5du2zwR8B&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005005488898046%7C_p_origin_prod%3A&amp;search_p4p_id=20260912085948577072255597880000865035_1</t>
-  </si>
-  <si>
-    <t>2.54mm PCB Pin headers</t>
-  </si>
-  <si>
-    <t>20x2p</t>
-  </si>
-  <si>
-    <t>25x2p</t>
   </si>
 </sst>
 </file>
@@ -817,21 +805,6 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13">
-        <v>1.04</v>
-      </c>
-      <c r="G13" t="s">
-        <v>35</v>
-      </c>
       <c r="H13" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
# 1 October 2026 - Starting the top case
</commit_message>
<xml_diff>
--- a/Keyboard BOM.xlsx
+++ b/Keyboard BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ac8f2ab3c324b6b/Documents/GitHub/Crazy-75/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="155" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CBF6BE5-0C6D-49F8-BE6B-15503DDA57F8}"/>
+  <xr:revisionPtr revIDLastSave="181" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41A76C5F-8628-4D38-8BF4-2B664B749FB8}"/>
   <bookViews>
-    <workbookView xWindow="20775" yWindow="4425" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
+    <workbookView xWindow="19680" yWindow="2550" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Part No.</t>
   </si>
@@ -62,12 +62,6 @@
     <t>.</t>
   </si>
   <si>
-    <t>Kailh Hot Plug Base</t>
-  </si>
-  <si>
-    <t>Kailh Hot-swappable PCB socket Hot Plug CPG151101S11 for Gateron Outemu Cherry MX Switches Mechanical Keyboard DIY wholesale</t>
-  </si>
-  <si>
     <t>https://fr.aliexpress.com/item/1005006105603269.html?spm=a2g0n.productlist.0.0.3858BhLlBhLlik&amp;browser_id=2269fcae49994bc495ac18d9a18a9643&amp;aff_trace_key=a9b6c8e739aa4a98a2d8e403b501ff28-1780918887469-07997-_DFhInr9&amp;aff_platform=msite&amp;m_page_id=v5mtilbuikgcav781a01db52ac211d721d5c185afe&amp;gclid=&amp;pdp_ext_f=%7B%22order%22%3A%22227%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.05%215.84%21%21%218.04%216.66%21%400b15834e17872048241487926e0cff%2112000035768903525%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3A5b165265%3Bm03_new_user%3A-29895%3BpisId%3A5000000215237127&amp;algo_pvid=b39dc535-db3c-4a87-95d6-ba503a4c97bf&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005006105603269%7C_p_origin_prod%3A</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
     <t>360 Degree Rotary Encoder EC11 With Push Button</t>
   </si>
   <si>
-    <t>EC11</t>
-  </si>
-  <si>
     <t>Switches</t>
   </si>
   <si>
@@ -144,13 +135,34 @@
   </si>
   <si>
     <t>USB cable</t>
+  </si>
+  <si>
+    <t>Quality solder</t>
+  </si>
+  <si>
+    <t>https://fr.aliexpress.com/item/1005005793344984.html?spm=a2g0o.productlist.main.21.8c8a71c4PRHiQa&amp;algo_pvid=f522a9a2-9f8c-4b3b-9379-39c4ef2a820d&amp;algo_exp_id=f522a9a2-9f8c-4b3b-9379-39c4ef2a820d-20&amp;pdp_ext_f=%7B%22order%22%3A%2248%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%214.25%213.91%21%21%214.70%214.32%21%402140f2bd17908666895603410e109b%2112000034374320916%21sea%21LU%218155715332%21X%211%210%21n_tag%3A-29911%3Bd%3Ae8fc6401%3Bm03_new_user%3A-29895&amp;curPageLogUid=S7v4FRbEFjS1&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005005793344984%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>Poron Gaskets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90x5x2mm </t>
+  </si>
+  <si>
+    <t>EC11 rotary encoder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kailh Hot-swappable PCB socket </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kailh style Hot-swappable PCB socket Hot Plug CPG151101S11 for Gateron Outemu Cherry MX Switches Mechanical Keyboard </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,6 +173,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Roboto"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF191919"/>
       <name val="Roboto"/>
       <charset val="238"/>
     </font>
@@ -185,9 +203,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5F0154-0866-430C-ACD5-87E79D9222E2}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -548,7 +567,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -568,13 +587,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="D2">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -583,7 +602,7 @@
         <v>7.91</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H2" t="s">
         <v>6</v>
@@ -594,10 +613,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H3" t="s">
         <v>6</v>
@@ -608,10 +627,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H4" t="s">
         <v>6</v>
@@ -622,10 +641,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E5">
         <v>100</v>
@@ -634,7 +653,7 @@
         <v>0.8</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H5" t="s">
         <v>6</v>
@@ -645,10 +664,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -657,7 +676,7 @@
         <v>4.3499999999999996</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
         <v>6</v>
@@ -668,10 +687,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -683,7 +702,7 @@
         <v>1.66</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H7" t="s">
         <v>6</v>
@@ -694,7 +713,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -706,7 +725,7 @@
         <v>3.61</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H8" t="s">
         <v>6</v>
@@ -717,22 +736,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H9" t="s">
         <v>6</v>
@@ -743,10 +762,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -758,7 +777,7 @@
         <v>2.62</v>
       </c>
       <c r="G10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H10" t="s">
         <v>6</v>
@@ -769,10 +788,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -784,7 +803,7 @@
         <v>1.92</v>
       </c>
       <c r="G11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H11" t="s">
         <v>6</v>
@@ -795,7 +814,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H12" t="s">
         <v>6</v>
@@ -805,7 +824,36 @@
       <c r="A13">
         <v>12</v>
       </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
       <c r="H13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14">
+        <v>3.91</v>
+      </c>
+      <c r="G14" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
24.10.2026 - PCB redesign
</commit_message>
<xml_diff>
--- a/Keyboard BOM.xlsx
+++ b/Keyboard BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ac8f2ab3c324b6b/Documents/GitHub/Crazy-75/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE8E815D-7878-4089-8C6A-9D25DD983282}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="8_{FCCC2E56-FDB1-4E02-ACF6-F81B5EFE9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{474906CF-4F07-449B-8940-5AA12D0DAC36}"/>
   <bookViews>
-    <workbookView xWindow="23700" yWindow="2145" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
+    <workbookView xWindow="2040" yWindow="2400" windowWidth="27300" windowHeight="15300" xr2:uid="{7E7D5457-AF9F-4A24-AB89-FCDAB66E2EA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="52">
   <si>
     <t>Part No.</t>
   </si>
@@ -186,6 +186,15 @@
   </si>
   <si>
     <t>25 + shipping</t>
+  </si>
+  <si>
+    <t>Frood RP2040 Pro Micro Controller</t>
+  </si>
+  <si>
+    <t>https://42keebs.eu/shop/parts/controllers/frood-rp2040-pro-micro-controller/?attribute_colour=Black</t>
+  </si>
+  <si>
+    <t>12.87 + 14.04 shipping</t>
   </si>
 </sst>
 </file>
@@ -575,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5F0154-0866-430C-ACD5-87E79D9222E2}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -967,6 +976,54 @@
         <v>6</v>
       </c>
     </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>